<commit_message>
Non-blocking concurrent dispatch, content-based reply matching, Android UI redesign
- Remove one-active-per-operator queue blocking — multiple requests now dispatch simultaneously
- Add payload-in-reply matching (phone/NID/IMEI appears in operator reply body) for disambiguation
- Import 144 training samples from xlsx files into reply-patterns.json
- Telegram bridge: group-membership authorization (empty authorizedUsers = any member can submit)
- Telegram bridge: seed notifiedTimeouts on restart to prevent re-notification
- Remove request ID from Telegram reply messages (internal detail, not for end users)
- Android app UI redesign: hero status indicator with pulse animation, live stats counters,
  collapsible gateway details, test request moved to Settings, branded app icon, toolbar menu
- Rewrite tests for concurrent dispatch model

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Training Data/Automation/NID-MS/1. GP/GP_NID_MS.xlsx
+++ b/Training Data/Automation/NID-MS/1. GP/GP_NID_MS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Automation\LCL\1. GP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\SMS_Automation\Training Data\Automation\NID-MS\1. GP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED780A2-8849-4385-BBD8-E586D51D6B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC54690E-0B1E-433D-A608-D27A4583BF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1770" yWindow="1770" windowWidth="17280" windowHeight="9984" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,26 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Request</t>
   </si>
   <si>
     <t>Reply</t>
-  </si>
-  <si>
-    <t>LRL 01327655002</t>
-  </si>
-  <si>
-    <t>MSISDN: 8801327655002
-LastActiveDateTime: 2026-06-10 18:32:49 06:00
-LACID: 46181
-CellID: 29713183
-Latitude: 22.45909
-Longitude: 89.83815
-Address: SARALIA,MORRELGANJ,MORRELGANJ,BAGERHAT
-CS Status: Idle
-Volte Status: not in VoLTE network [GP]</t>
   </si>
 </sst>
 </file>
@@ -372,16 +358,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="2" max="2" width="27.28515625" customWidth="1"/>
-    <col min="3" max="3" width="44.85546875" customWidth="1"/>
+    <col min="2" max="2" width="27.26171875" customWidth="1"/>
+    <col min="3" max="3" width="44.83984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2">
-        <v>1</v>
-      </c>
+    <row r="1" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -389,80 +373,76 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="150" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="2">
         <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>